<commit_message>
add balanced metrics to base run
</commit_message>
<xml_diff>
--- a/dataset_agreed/saved_models/baserun/greyscale_testrun_run_1/epoch_100/per_file_predictions_epoch_100.xlsx
+++ b/dataset_agreed/saved_models/baserun/greyscale_testrun_run_1/epoch_100/per_file_predictions_epoch_100.xlsx
@@ -1282,7 +1282,7 @@
     <t>0.1034,0.0000,0.9410,0.0000</t>
   </si>
   <si>
-    <t>0.4343,0.0001,0.6162,0.0000</t>
+    <t>0.4344,0.0001,0.6162,0.0000</t>
   </si>
   <si>
     <t>0.0000,0.0000,1.0000,0.0000</t>
@@ -1468,7 +1468,7 @@
     <t>0.9760,0.0282,0.0017,0.0009</t>
   </si>
   <si>
-    <t>0.9246,0.0450,0.0140,0.0060</t>
+    <t>0.9246,0.0449,0.0140,0.0060</t>
   </si>
   <si>
     <t>0.9448,0.0374,0.0032,0.0015</t>

</xml_diff>